<commit_message>
Add budget tiers and pace-based itinerary
Replace numeric daily budget input with selectable budget tiers and add explicit travel pace selection in the CLI. Map budget tiers to estimated daily/total budgets in UserProfile.__post_init__, and update printed user profile to show tier and estimated daily cost. Update preference collector options (interests list and budget labels) to match new simplified categories. Adjust POI ranking logic to consider budget_tier (with stronger boosts/penalties), incorporate pace-aware duration scoring, and limit daily POI count based on selected pace. Minor CLI/print UX tweaks and updated binary assets (POI embeddings, spreadsheet, and compiled module).
</commit_message>
<xml_diff>
--- a/Cairo_Giza_Final_Verified_POIs.xlsx
+++ b/Cairo_Giza_Final_Verified_POIs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Abraam Refaat\Documents\GitHub\Nile-Quest---Graduation-Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59E33C59-6EED-465E-A60C-033F5B17F8A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20D1CE37-4E72-4A7B-A981-6B84862FDE33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1205" uniqueCount="412">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1212" uniqueCount="415">
   <si>
     <t>Name</t>
   </si>
@@ -1256,13 +1256,22 @@
   </si>
   <si>
     <t>Indoor/Outdoor</t>
+  </si>
+  <si>
+    <t>Saladin Citadel</t>
+  </si>
+  <si>
+    <t>30.0287° N, 31.2597° E</t>
+  </si>
+  <si>
+    <t>Citadel</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1277,6 +1286,18 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1314,11 +1335,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1623,7 +1646,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H172"/>
+  <dimension ref="A1:H173"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -6023,7 +6046,34 @@
         <v>411</v>
       </c>
     </row>
+    <row r="173" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A173" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="B173" t="s">
+        <v>413</v>
+      </c>
+      <c r="C173" t="s">
+        <v>323</v>
+      </c>
+      <c r="D173" t="s">
+        <v>414</v>
+      </c>
+      <c r="E173" t="s">
+        <v>379</v>
+      </c>
+      <c r="F173" s="3">
+        <v>500</v>
+      </c>
+      <c r="G173" t="s">
+        <v>380</v>
+      </c>
+      <c r="H173" t="s">
+        <v>411</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>